<commit_message>
Rodada 2: planilhas preenchidas e fichas C1-C10
</commit_message>
<xml_diff>
--- a/data/modelos/lesoes_suspensoes_2026.xlsx
+++ b/data/modelos/lesoes_suspensoes_2026.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEIA" sheetId="1" r:id="Reee00b8b0b4649d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesoes" sheetId="2" r:id="Redb4e3f1bc954a03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suspensoes" sheetId="3" r:id="R73816626c54c460b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEIA" sheetId="1" r:id="R6fd90532a0184c7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesoes" sheetId="2" r:id="R85ed022b91904191"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suspensoes" sheetId="3" r:id="R1e76d32f742d44fc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,7 +15,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="11">
+  <x:fonts count="15">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -78,8 +78,36 @@
       <x:family val="2"/>
       <x:scheme val="minor"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF222222"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+      <x:family val="2"/>
+      <x:scheme val="minor"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF222222"/>
+      <x:name val="Arial"/>
+      <x:family val="2"/>
+      <x:scheme val="minor"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -89,6 +117,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFDDEBF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -104,7 +142,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="26">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -138,6 +176,37 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -1040,83 +1109,55 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="70" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="44" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="76" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="3" t="str">
+    <x:row r="1" ht="18" customHeight="1">
+      <x:c r="A1" s="24" t="str">
         <x:v>clube</x:v>
       </x:c>
-      <x:c r="B1" s="3" t="str">
+      <x:c r="B1" s="24" t="str">
         <x:v>nome_comum</x:v>
       </x:c>
-      <x:c r="C1" s="3" t="str">
+      <x:c r="C1" s="24" t="str">
         <x:v>competicao</x:v>
       </x:c>
-      <x:c r="D1" s="3" t="str">
+      <x:c r="D1" s="24" t="str">
         <x:v>jogos</x:v>
       </x:c>
-      <x:c r="E1" s="3" t="str">
+      <x:c r="E1" s="24" t="str">
         <x:v>motivo</x:v>
       </x:c>
-      <x:c r="F1" s="3" t="str">
+      <x:c r="F1" s="24" t="str">
         <x:v>fonte</x:v>
       </x:c>
-      <x:c r="G1" t="str">
+      <x:c r="G1" s="25" t="str">
         <x:v>atualizado</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="18" customHeight="1">
-      <x:c r="A2" s="14" t="str">
-        <x:v>Remo</x:v>
-      </x:c>
-      <x:c r="B2" s="14" t="str">
-        <x:v>Nico Ferreira</x:v>
-      </x:c>
-      <x:c r="C2" s="14" t="str">
-        <x:v>Série A</x:v>
-      </x:c>
-      <x:c r="D2" s="14" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E2" s="14" t="str">
-        <x:v>punição remanescente da Série B 2025</x:v>
-      </x:c>
-      <x:c r="F2" s="14" t="str">
-        <x:v>https://ge.globo.com/cartola/noticia/2026/01/28/cartola-2026-veja-suspensos-lesionados-e-escalacoes-provaveis-da-primeira-rodada-do-brasileirao.ghtml</x:v>
-      </x:c>
-      <x:c r="G2" s="14" t="str">
-        <x:v>2026-10-20</x:v>
-      </x:c>
+      <x:c r="A2" s="14"/>
+      <x:c r="B2" s="14"/>
+      <x:c r="C2" s="14"/>
+      <x:c r="D2" s="14"/>
+      <x:c r="E2" s="14"/>
+      <x:c r="F2" s="14"/>
+      <x:c r="G2" s="14"/>
     </x:row>
     <x:row r="3" ht="18" customHeight="1">
-      <x:c r="A3" s="14" t="str">
-        <x:v>Remo</x:v>
-      </x:c>
-      <x:c r="B3" s="14" t="str">
-        <x:v>Diego Hernández</x:v>
-      </x:c>
-      <x:c r="C3" s="14" t="str">
-        <x:v>Série A</x:v>
-      </x:c>
-      <x:c r="D3" s="14" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E3" s="14" t="str">
-        <x:v>punição remanescente da Série B 2025</x:v>
-      </x:c>
-      <x:c r="F3" s="14" t="str">
-        <x:v>https://ge.globo.com/cartola/noticia/2026/01/28/cartola-2026-veja-suspensos-lesionados-e-escalacoes-provaveis-da-primeira-rodada-do-brasileirao.ghtml</x:v>
-      </x:c>
-      <x:c r="G3" s="14" t="str">
-        <x:v>2026-10-20</x:v>
-      </x:c>
+      <x:c r="A3" s="14"/>
+      <x:c r="B3" s="14"/>
+      <x:c r="C3" s="14"/>
+      <x:c r="D3" s="14"/>
+      <x:c r="E3" s="14"/>
+      <x:c r="F3" s="14"/>
+      <x:c r="G3" s="14"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>